<commit_message>
test: login without credentials and validate the error message
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>CT</t>
   </si>
@@ -59,6 +59,60 @@
   </si>
   <si>
     <t>TESTE</t>
+  </si>
+  <si>
+    <t>002</t>
+  </si>
+  <si>
+    <t>003</t>
+  </si>
+  <si>
+    <t>004</t>
+  </si>
+  <si>
+    <t>005</t>
+  </si>
+  <si>
+    <t>006</t>
+  </si>
+  <si>
+    <t>007</t>
+  </si>
+  <si>
+    <t>008</t>
+  </si>
+  <si>
+    <t>009</t>
+  </si>
+  <si>
+    <t>010</t>
+  </si>
+  <si>
+    <t>011</t>
+  </si>
+  <si>
+    <t>012</t>
+  </si>
+  <si>
+    <t>013</t>
+  </si>
+  <si>
+    <t>014</t>
+  </si>
+  <si>
+    <t>015</t>
+  </si>
+  <si>
+    <t>016</t>
+  </si>
+  <si>
+    <t>017</t>
+  </si>
+  <si>
+    <t>018</t>
+  </si>
+  <si>
+    <t>019</t>
   </si>
 </sst>
 </file>
@@ -433,20 +487,22 @@
       <c r="V2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
+      <c r="A3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
@@ -457,20 +513,22 @@
       <c r="V3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
+      <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
@@ -481,20 +539,22 @@
       <c r="V4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
+      <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
@@ -505,20 +565,22 @@
       <c r="V5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
+      <c r="A6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
@@ -529,20 +591,22 @@
       <c r="V6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
@@ -553,20 +617,22 @@
       <c r="V7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="4"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
@@ -577,20 +643,22 @@
       <c r="V8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
+      <c r="A9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
@@ -601,20 +669,22 @@
       <c r="V9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
+      <c r="A10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
@@ -625,20 +695,22 @@
       <c r="V10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
+      <c r="A11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
@@ -649,20 +721,22 @@
       <c r="V11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
+      <c r="A12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
       <c r="O12" s="4"/>
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
@@ -673,20 +747,22 @@
       <c r="V12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
+      <c r="A13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
       <c r="O13" s="4"/>
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
@@ -697,20 +773,22 @@
       <c r="V13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
+      <c r="A14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
       <c r="O14" s="4"/>
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
@@ -721,20 +799,22 @@
       <c r="V14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
+      <c r="A15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
       <c r="O15" s="4"/>
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
@@ -745,20 +825,22 @@
       <c r="V15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
+      <c r="A16" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
       <c r="O16" s="4"/>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
@@ -769,20 +851,22 @@
       <c r="V16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
+      <c r="A17" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
       <c r="O17" s="4"/>
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
@@ -793,20 +877,22 @@
       <c r="V17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
+      <c r="A18" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
@@ -817,20 +903,22 @@
       <c r="V18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4"/>
+      <c r="A19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
       <c r="O19" s="4"/>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
@@ -841,20 +929,22 @@
       <c r="V19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
+      <c r="A20" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
       <c r="O20" s="4"/>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
@@ -24096,30 +24186,6 @@
       <c r="U988" s="4"/>
       <c r="V988" s="4"/>
     </row>
-    <row r="989">
-      <c r="A989" s="4"/>
-      <c r="B989" s="4"/>
-      <c r="C989" s="4"/>
-      <c r="D989" s="4"/>
-      <c r="E989" s="4"/>
-      <c r="F989" s="4"/>
-      <c r="G989" s="4"/>
-      <c r="H989" s="4"/>
-      <c r="I989" s="4"/>
-      <c r="J989" s="4"/>
-      <c r="K989" s="4"/>
-      <c r="L989" s="4"/>
-      <c r="M989" s="4"/>
-      <c r="N989" s="4"/>
-      <c r="O989" s="4"/>
-      <c r="P989" s="4"/>
-      <c r="Q989" s="4"/>
-      <c r="R989" s="4"/>
-      <c r="S989" s="4"/>
-      <c r="T989" s="4"/>
-      <c r="U989" s="4"/>
-      <c r="V989" s="4"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
test: validate successful logout
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
   <si>
     <t>CT</t>
   </si>
@@ -516,8 +516,12 @@
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>

</xml_diff>

<commit_message>
test: validate sort by name ascending
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
   <si>
     <t>CT</t>
   </si>
@@ -22,7 +22,7 @@
     <t xml:space="preserve">PASSWORD  </t>
   </si>
   <si>
-    <t>NAME</t>
+    <t>SORT</t>
   </si>
   <si>
     <t>FIRSTNAME</t>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>004</t>
+  </si>
+  <si>
+    <t>NAME_ASCENDING</t>
   </si>
   <si>
     <t>005</t>
@@ -395,6 +398,7 @@
   <cols>
     <col customWidth="1" min="2" max="2" width="19.63"/>
     <col customWidth="1" min="3" max="3" width="21.63"/>
+    <col customWidth="1" min="4" max="4" width="29.13"/>
     <col customWidth="1" min="5" max="5" width="18.38"/>
     <col customWidth="1" min="6" max="6" width="17.13"/>
     <col customWidth="1" min="7" max="7" width="16.0"/>
@@ -414,7 +418,7 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -548,7 +552,9 @@
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+      <c r="D5" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -570,7 +576,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -596,7 +602,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -622,7 +628,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -648,7 +654,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -674,7 +680,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -700,7 +706,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -726,7 +732,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -752,7 +758,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -778,7 +784,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -804,7 +810,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -830,7 +836,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -856,7 +862,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -882,7 +888,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -908,7 +914,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -934,7 +940,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>

</xml_diff>

<commit_message>
test: validate sort by name descending
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testData.xlsx
+++ b/src/test/resources/testData/testData.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
   <si>
     <t>CT</t>
   </si>
@@ -76,10 +76,19 @@
     <t>005</t>
   </si>
   <si>
+    <t>NAME_DESCENDING</t>
+  </si>
+  <si>
     <t>006</t>
   </si>
   <si>
+    <t>PRICE_ASCENDING</t>
+  </si>
+  <si>
     <t>007</t>
+  </si>
+  <si>
+    <t>PRICE_DESCENDING</t>
   </si>
   <si>
     <t>008</t>
@@ -398,7 +407,7 @@
   <cols>
     <col customWidth="1" min="2" max="2" width="19.63"/>
     <col customWidth="1" min="3" max="3" width="21.63"/>
-    <col customWidth="1" min="4" max="4" width="29.13"/>
+    <col customWidth="1" min="4" max="4" width="31.38"/>
     <col customWidth="1" min="5" max="5" width="18.38"/>
     <col customWidth="1" min="6" max="6" width="17.13"/>
     <col customWidth="1" min="7" max="7" width="16.0"/>
@@ -580,7 +589,9 @@
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="D6" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -602,11 +613,13 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
+      <c r="D7" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -628,11 +641,13 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
+      <c r="D8" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -654,7 +669,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -680,7 +695,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -706,7 +721,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -732,7 +747,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -758,7 +773,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -784,7 +799,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -810,7 +825,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -836,7 +851,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -862,7 +877,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -888,7 +903,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -914,7 +929,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -940,7 +955,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>

</xml_diff>